<commit_message>
Update excel sheet v3
</commit_message>
<xml_diff>
--- a/STAIX2026/assets/Poster-Presentation-Label-Assignment.xlsx
+++ b/STAIX2026/assets/Poster-Presentation-Label-Assignment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tracyke/Dropbox/Mac (2)/Documents/2026/STAI-X conference/Poster session/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21276E5-A52B-1040-B89A-1D24086F1E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07E6659-BFEC-D046-878E-7CCBF2DA6420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9000" yWindow="4080" windowWidth="38400" windowHeight="19240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="500" windowWidth="38400" windowHeight="19240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assignment" sheetId="7" r:id="rId1"/>
@@ -600,7 +600,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
@@ -617,6 +617,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -635,13 +638,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1171,7 +1167,7 @@
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="17" t="s">
         <v>131</v>
       </c>
     </row>
@@ -1188,7 +1184,7 @@
       <c r="E3" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="15"/>
+      <c r="I3" s="18"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A4" s="1">
@@ -1206,7 +1202,7 @@
       <c r="E4" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="15"/>
+      <c r="I4" s="18"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A5" s="2">
@@ -1221,7 +1217,7 @@
       <c r="E5" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="15"/>
+      <c r="I5" s="18"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A6" s="2">
@@ -1236,7 +1232,7 @@
       <c r="E6" t="s">
         <v>4</v>
       </c>
-      <c r="I6" s="15"/>
+      <c r="I6" s="18"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A7" s="3">
@@ -1251,7 +1247,7 @@
       <c r="E7" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="15"/>
+      <c r="I7" s="18"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A8" s="3">
@@ -1266,7 +1262,7 @@
       <c r="E8" t="s">
         <v>4</v>
       </c>
-      <c r="I8" s="15"/>
+      <c r="I8" s="18"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A9" s="3">
@@ -1281,7 +1277,7 @@
       <c r="E9" t="s">
         <v>4</v>
       </c>
-      <c r="I9" s="15"/>
+      <c r="I9" s="18"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A10" s="3">
@@ -1296,7 +1292,7 @@
       <c r="E10" t="s">
         <v>4</v>
       </c>
-      <c r="I10" s="15"/>
+      <c r="I10" s="18"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A11" s="1">
@@ -1311,7 +1307,7 @@
       <c r="E11" t="s">
         <v>4</v>
       </c>
-      <c r="I11" s="15"/>
+      <c r="I11" s="18"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A12" s="1">
@@ -1329,7 +1325,7 @@
       <c r="E12" t="s">
         <v>4</v>
       </c>
-      <c r="I12" s="15"/>
+      <c r="I12" s="18"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A13" s="3">
@@ -1344,7 +1340,7 @@
       <c r="E13" t="s">
         <v>4</v>
       </c>
-      <c r="I13" s="15"/>
+      <c r="I13" s="18"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A14" s="3">
@@ -1359,7 +1355,7 @@
       <c r="E14" t="s">
         <v>4</v>
       </c>
-      <c r="I14" s="15"/>
+      <c r="I14" s="18"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A15" s="3">
@@ -1374,7 +1370,7 @@
       <c r="E15" t="s">
         <v>4</v>
       </c>
-      <c r="I15" s="15"/>
+      <c r="I15" s="18"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A16" s="3">
@@ -1389,7 +1385,7 @@
       <c r="E16" t="s">
         <v>4</v>
       </c>
-      <c r="I16" s="15"/>
+      <c r="I16" s="18"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A17" s="3">
@@ -1404,7 +1400,7 @@
       <c r="E17" t="s">
         <v>4</v>
       </c>
-      <c r="I17" s="15"/>
+      <c r="I17" s="18"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
@@ -1419,7 +1415,7 @@
       <c r="E18" t="s">
         <v>8</v>
       </c>
-      <c r="I18" s="15"/>
+      <c r="I18" s="18"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A19" s="1">
@@ -1434,7 +1430,7 @@
       <c r="E19" t="s">
         <v>8</v>
       </c>
-      <c r="I19" s="15"/>
+      <c r="I19" s="18"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A20" s="1">
@@ -1449,7 +1445,7 @@
       <c r="E20" t="s">
         <v>8</v>
       </c>
-      <c r="I20" s="15"/>
+      <c r="I20" s="18"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A21" s="2">
@@ -1464,7 +1460,7 @@
       <c r="E21" t="s">
         <v>8</v>
       </c>
-      <c r="I21" s="15"/>
+      <c r="I21" s="18"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A22" s="3">
@@ -1479,7 +1475,7 @@
       <c r="E22" t="s">
         <v>8</v>
       </c>
-      <c r="I22" s="15"/>
+      <c r="I22" s="18"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A23" s="3">
@@ -1494,7 +1490,7 @@
       <c r="E23" t="s">
         <v>8</v>
       </c>
-      <c r="I23" s="15"/>
+      <c r="I23" s="18"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A24" s="3">
@@ -1509,7 +1505,7 @@
       <c r="E24" t="s">
         <v>8</v>
       </c>
-      <c r="I24" s="15"/>
+      <c r="I24" s="18"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A25" s="3">
@@ -1527,7 +1523,7 @@
       <c r="E25" t="s">
         <v>8</v>
       </c>
-      <c r="I25" s="15"/>
+      <c r="I25" s="18"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A26" s="2">
@@ -1542,7 +1538,7 @@
       <c r="E26" t="s">
         <v>8</v>
       </c>
-      <c r="I26" s="15"/>
+      <c r="I26" s="18"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A27" s="1">
@@ -1560,7 +1556,7 @@
       <c r="E27" t="s">
         <v>8</v>
       </c>
-      <c r="I27" s="15"/>
+      <c r="I27" s="18"/>
     </row>
     <row r="28" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1">
@@ -1575,7 +1571,7 @@
       <c r="E28" t="s">
         <v>8</v>
       </c>
-      <c r="I28" s="15"/>
+      <c r="I28" s="18"/>
     </row>
     <row r="29" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="3">
@@ -1593,7 +1589,7 @@
       <c r="E29" t="s">
         <v>8</v>
       </c>
-      <c r="I29" s="15"/>
+      <c r="I29" s="18"/>
     </row>
     <row r="30" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="3">
@@ -1608,7 +1604,7 @@
       <c r="E30" t="s">
         <v>8</v>
       </c>
-      <c r="I30" s="15"/>
+      <c r="I30" s="18"/>
     </row>
     <row r="31" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="3">
@@ -1623,7 +1619,7 @@
       <c r="E31" t="s">
         <v>8</v>
       </c>
-      <c r="I31" s="15"/>
+      <c r="I31" s="18"/>
     </row>
     <row r="32" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="3">
@@ -1638,7 +1634,7 @@
       <c r="E32" t="s">
         <v>8</v>
       </c>
-      <c r="I32" s="15"/>
+      <c r="I32" s="18"/>
     </row>
     <row r="33" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="2">
@@ -1653,7 +1649,7 @@
       <c r="E33" t="s">
         <v>8</v>
       </c>
-      <c r="I33" s="15"/>
+      <c r="I33" s="18"/>
     </row>
     <row r="34" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="3">
@@ -1668,7 +1664,7 @@
       <c r="E34" t="s">
         <v>14</v>
       </c>
-      <c r="I34" s="15"/>
+      <c r="I34" s="18"/>
     </row>
     <row r="35" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="1">
@@ -1686,7 +1682,7 @@
       <c r="E35" t="s">
         <v>14</v>
       </c>
-      <c r="I35" s="15"/>
+      <c r="I35" s="18"/>
     </row>
     <row r="36" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="1">
@@ -1701,7 +1697,7 @@
       <c r="E36" t="s">
         <v>14</v>
       </c>
-      <c r="I36" s="15"/>
+      <c r="I36" s="18"/>
     </row>
     <row r="37" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="1">
@@ -1716,7 +1712,7 @@
       <c r="E37" t="s">
         <v>14</v>
       </c>
-      <c r="I37" s="15"/>
+      <c r="I37" s="18"/>
     </row>
     <row r="38" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="2">
@@ -1731,7 +1727,7 @@
       <c r="E38" t="s">
         <v>14</v>
       </c>
-      <c r="I38" s="15"/>
+      <c r="I38" s="18"/>
     </row>
     <row r="39" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="2">
@@ -1746,7 +1742,7 @@
       <c r="E39" t="s">
         <v>14</v>
       </c>
-      <c r="I39" s="15"/>
+      <c r="I39" s="18"/>
     </row>
     <row r="40" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="3">
@@ -1764,7 +1760,7 @@
       <c r="E40" t="s">
         <v>14</v>
       </c>
-      <c r="I40" s="15"/>
+      <c r="I40" s="18"/>
     </row>
     <row r="41" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="3">
@@ -1779,7 +1775,7 @@
       <c r="E41" t="s">
         <v>14</v>
       </c>
-      <c r="I41" s="15"/>
+      <c r="I41" s="18"/>
     </row>
     <row r="42" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="3">
@@ -1794,7 +1790,7 @@
       <c r="E42" t="s">
         <v>14</v>
       </c>
-      <c r="I42" s="15"/>
+      <c r="I42" s="18"/>
     </row>
     <row r="43" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="3">
@@ -1809,38 +1805,35 @@
       <c r="E43" t="s">
         <v>14</v>
       </c>
-      <c r="I43" s="15"/>
+      <c r="I43" s="18"/>
     </row>
     <row r="44" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A44" s="23">
+      <c r="A44" s="3">
         <v>37</v>
       </c>
-      <c r="B44" s="23" t="s">
+      <c r="B44" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C44" s="24"/>
       <c r="D44" s="8">
         <v>43</v>
       </c>
-      <c r="E44" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="F44" s="24"/>
-      <c r="G44" s="24"/>
-      <c r="I44" s="15"/>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="I44" s="18"/>
     </row>
     <row r="45" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="25"/>
-      <c r="B45" s="25"/>
-      <c r="C45" s="25"/>
-      <c r="D45" s="26">
+      <c r="A45" s="15"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="16">
         <v>44</v>
       </c>
-      <c r="E45" s="25"/>
-      <c r="F45" s="25"/>
-      <c r="G45" s="25"/>
-      <c r="H45" s="25"/>
-      <c r="I45" s="16"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="15"/>
+      <c r="H45" s="15"/>
+      <c r="I45" s="19"/>
     </row>
     <row r="46" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="3">
@@ -1855,7 +1848,7 @@
       <c r="E46" t="s">
         <v>14</v>
       </c>
-      <c r="I46" s="17" t="s">
+      <c r="I46" s="20" t="s">
         <v>132</v>
       </c>
     </row>
@@ -1872,7 +1865,7 @@
       <c r="E47" t="s">
         <v>14</v>
       </c>
-      <c r="I47" s="18"/>
+      <c r="I47" s="21"/>
     </row>
     <row r="48" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="1">
@@ -1887,13 +1880,13 @@
       <c r="E48" t="s">
         <v>14</v>
       </c>
-      <c r="I48" s="18"/>
+      <c r="I48" s="21"/>
     </row>
     <row r="49" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="1">
         <v>63</v>
       </c>
-      <c r="B49" s="20" t="s">
+      <c r="B49" s="14" t="s">
         <v>140</v>
       </c>
       <c r="D49" s="8">
@@ -1902,7 +1895,7 @@
       <c r="E49" t="s">
         <v>14</v>
       </c>
-      <c r="I49" s="18"/>
+      <c r="I49" s="21"/>
     </row>
     <row r="50" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="1">
@@ -1917,7 +1910,7 @@
       <c r="E50" t="s">
         <v>14</v>
       </c>
-      <c r="I50" s="18"/>
+      <c r="I50" s="21"/>
     </row>
     <row r="51" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="1">
@@ -1932,7 +1925,7 @@
       <c r="E51" t="s">
         <v>14</v>
       </c>
-      <c r="I51" s="18"/>
+      <c r="I51" s="21"/>
     </row>
     <row r="52" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="2">
@@ -1947,7 +1940,7 @@
       <c r="E52" t="s">
         <v>14</v>
       </c>
-      <c r="I52" s="18"/>
+      <c r="I52" s="21"/>
     </row>
     <row r="53" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="2">
@@ -1962,7 +1955,7 @@
       <c r="E53" t="s">
         <v>14</v>
       </c>
-      <c r="I53" s="18"/>
+      <c r="I53" s="21"/>
     </row>
     <row r="54" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="3">
@@ -1980,7 +1973,7 @@
       <c r="E54" t="s">
         <v>14</v>
       </c>
-      <c r="I54" s="18"/>
+      <c r="I54" s="21"/>
     </row>
     <row r="55" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="3">
@@ -1995,7 +1988,7 @@
       <c r="E55" t="s">
         <v>14</v>
       </c>
-      <c r="I55" s="18"/>
+      <c r="I55" s="21"/>
     </row>
     <row r="56" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="3">
@@ -2010,7 +2003,7 @@
       <c r="E56" t="s">
         <v>14</v>
       </c>
-      <c r="I56" s="18"/>
+      <c r="I56" s="21"/>
     </row>
     <row r="57" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="3">
@@ -2025,7 +2018,7 @@
       <c r="E57" t="s">
         <v>14</v>
       </c>
-      <c r="I57" s="18"/>
+      <c r="I57" s="21"/>
     </row>
     <row r="58" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="3">
@@ -2040,7 +2033,7 @@
       <c r="E58" t="s">
         <v>14</v>
       </c>
-      <c r="I58" s="18"/>
+      <c r="I58" s="21"/>
     </row>
     <row r="59" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="3">
@@ -2055,25 +2048,22 @@
       <c r="E59" t="s">
         <v>14</v>
       </c>
-      <c r="I59" s="18"/>
+      <c r="I59" s="21"/>
     </row>
     <row r="60" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="3">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C60" t="s">
-        <v>68</v>
+        <v>144</v>
       </c>
       <c r="D60" s="8">
         <v>59</v>
       </c>
       <c r="E60" t="s">
-        <v>14</v>
-      </c>
-      <c r="I60" s="18"/>
+        <v>6</v>
+      </c>
+      <c r="I60" s="21"/>
     </row>
     <row r="61" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="1">
@@ -2091,7 +2081,7 @@
       <c r="E61" t="s">
         <v>14</v>
       </c>
-      <c r="I61" s="18"/>
+      <c r="I61" s="21"/>
     </row>
     <row r="62" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="3">
@@ -2106,7 +2096,7 @@
       <c r="E62" t="s">
         <v>14</v>
       </c>
-      <c r="I62" s="18"/>
+      <c r="I62" s="21"/>
     </row>
     <row r="63" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="3">
@@ -2121,13 +2111,13 @@
       <c r="E63" t="s">
         <v>14</v>
       </c>
-      <c r="I63" s="18"/>
+      <c r="I63" s="21"/>
     </row>
     <row r="64" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="3">
         <v>34</v>
       </c>
-      <c r="B64" s="21" t="s">
+      <c r="B64" s="3" t="s">
         <v>145</v>
       </c>
       <c r="D64" s="8">
@@ -2136,7 +2126,7 @@
       <c r="E64" t="s">
         <v>6</v>
       </c>
-      <c r="I64" s="18"/>
+      <c r="I64" s="21"/>
     </row>
     <row r="65" spans="1:9" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="3">
@@ -2154,7 +2144,7 @@
       <c r="E65" t="s">
         <v>6</v>
       </c>
-      <c r="I65" s="18"/>
+      <c r="I65" s="21"/>
     </row>
     <row r="66" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="3">
@@ -2169,7 +2159,7 @@
       <c r="E66" t="s">
         <v>6</v>
       </c>
-      <c r="I66" s="18"/>
+      <c r="I66" s="21"/>
     </row>
     <row r="67" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="3">
@@ -2184,7 +2174,7 @@
       <c r="E67" t="s">
         <v>6</v>
       </c>
-      <c r="I67" s="18"/>
+      <c r="I67" s="21"/>
     </row>
     <row r="68" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="3">
@@ -2199,7 +2189,7 @@
       <c r="E68" t="s">
         <v>6</v>
       </c>
-      <c r="I68" s="18"/>
+      <c r="I68" s="21"/>
     </row>
     <row r="69" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A69" s="2">
@@ -2214,7 +2204,7 @@
       <c r="E69" t="s">
         <v>6</v>
       </c>
-      <c r="I69" s="18"/>
+      <c r="I69" s="21"/>
     </row>
     <row r="70" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A70" s="2">
@@ -2229,7 +2219,7 @@
       <c r="E70" t="s">
         <v>6</v>
       </c>
-      <c r="I70" s="18"/>
+      <c r="I70" s="21"/>
     </row>
     <row r="71" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="3">
@@ -2244,7 +2234,7 @@
       <c r="E71" t="s">
         <v>6</v>
       </c>
-      <c r="I71" s="18"/>
+      <c r="I71" s="21"/>
     </row>
     <row r="72" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A72" s="3">
@@ -2259,7 +2249,7 @@
       <c r="E72" t="s">
         <v>6</v>
       </c>
-      <c r="I72" s="18"/>
+      <c r="I72" s="21"/>
     </row>
     <row r="73" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="3">
@@ -2274,7 +2264,7 @@
       <c r="E73" t="s">
         <v>6</v>
       </c>
-      <c r="I73" s="18"/>
+      <c r="I73" s="21"/>
     </row>
     <row r="74" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A74" s="1">
@@ -2292,7 +2282,7 @@
       <c r="E74" t="s">
         <v>6</v>
       </c>
-      <c r="I74" s="18"/>
+      <c r="I74" s="21"/>
     </row>
     <row r="75" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A75" s="3">
@@ -2307,7 +2297,7 @@
       <c r="E75" t="s">
         <v>6</v>
       </c>
-      <c r="I75" s="18"/>
+      <c r="I75" s="21"/>
     </row>
     <row r="76" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A76" s="3">
@@ -2322,7 +2312,7 @@
       <c r="E76" t="s">
         <v>6</v>
       </c>
-      <c r="I76" s="18"/>
+      <c r="I76" s="21"/>
     </row>
     <row r="77" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A77" s="3">
@@ -2337,7 +2327,7 @@
       <c r="E77" t="s">
         <v>6</v>
       </c>
-      <c r="I77" s="18"/>
+      <c r="I77" s="21"/>
     </row>
     <row r="78" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A78" s="3">
@@ -2352,7 +2342,7 @@
       <c r="E78" t="s">
         <v>6</v>
       </c>
-      <c r="I78" s="18"/>
+      <c r="I78" s="21"/>
     </row>
     <row r="79" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A79" s="3">
@@ -2367,7 +2357,7 @@
       <c r="E79" t="s">
         <v>6</v>
       </c>
-      <c r="I79" s="18"/>
+      <c r="I79" s="21"/>
     </row>
     <row r="80" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A80" s="3">
@@ -2382,7 +2372,7 @@
       <c r="E80" t="s">
         <v>6</v>
       </c>
-      <c r="I80" s="18"/>
+      <c r="I80" s="21"/>
     </row>
     <row r="81" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A81" s="2">
@@ -2397,7 +2387,7 @@
       <c r="E81" t="s">
         <v>4</v>
       </c>
-      <c r="I81" s="18"/>
+      <c r="I81" s="21"/>
     </row>
     <row r="82" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A82" s="3">
@@ -2412,7 +2402,7 @@
       <c r="E82" t="s">
         <v>6</v>
       </c>
-      <c r="I82" s="18"/>
+      <c r="I82" s="21"/>
     </row>
     <row r="83" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A83" s="3">
@@ -2427,7 +2417,7 @@
       <c r="E83" t="s">
         <v>14</v>
       </c>
-      <c r="I83" s="18"/>
+      <c r="I83" s="21"/>
     </row>
     <row r="84" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A84" s="3">
@@ -2442,7 +2432,7 @@
       <c r="E84" t="s">
         <v>14</v>
       </c>
-      <c r="I84" s="18"/>
+      <c r="I84" s="21"/>
     </row>
     <row r="85" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A85" s="3">
@@ -2460,13 +2450,13 @@
       <c r="E85" t="s">
         <v>14</v>
       </c>
-      <c r="I85" s="18"/>
+      <c r="I85" s="21"/>
     </row>
     <row r="86" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A86" s="3">
         <v>56</v>
       </c>
-      <c r="B86" s="21" t="s">
+      <c r="B86" s="3" t="s">
         <v>143</v>
       </c>
       <c r="D86" s="8">
@@ -2475,7 +2465,7 @@
       <c r="E86" t="s">
         <v>1</v>
       </c>
-      <c r="I86" s="18"/>
+      <c r="I86" s="21"/>
     </row>
     <row r="87" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A87" s="6"/>
@@ -2490,7 +2480,7 @@
       <c r="F87" s="6"/>
       <c r="G87" s="6"/>
       <c r="H87" s="6"/>
-      <c r="I87" s="19"/>
+      <c r="I87" s="22"/>
     </row>
     <row r="88" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A88" s="3">
@@ -2505,7 +2495,7 @@
       <c r="E88" t="s">
         <v>6</v>
       </c>
-      <c r="I88" s="14" t="s">
+      <c r="I88" s="17" t="s">
         <v>133</v>
       </c>
     </row>
@@ -2522,14 +2512,14 @@
       <c r="E89" t="s">
         <v>6</v>
       </c>
-      <c r="I89" s="15"/>
+      <c r="I89" s="18"/>
     </row>
     <row r="90" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A90" s="3">
-        <v>50</v>
-      </c>
-      <c r="B90" s="22" t="s">
-        <v>144</v>
+      <c r="A90" s="1">
+        <v>24</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="D90" s="8">
         <v>91</v>
@@ -2537,7 +2527,7 @@
       <c r="E90" t="s">
         <v>6</v>
       </c>
-      <c r="I90" s="15"/>
+      <c r="I90" s="18"/>
     </row>
     <row r="91" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A91" s="1">
@@ -2555,7 +2545,7 @@
       <c r="E91" t="s">
         <v>6</v>
       </c>
-      <c r="I91" s="15"/>
+      <c r="I91" s="18"/>
     </row>
     <row r="92" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A92" s="1">
@@ -2573,7 +2563,7 @@
       <c r="E92" t="s">
         <v>6</v>
       </c>
-      <c r="I92" s="15"/>
+      <c r="I92" s="18"/>
     </row>
     <row r="93" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A93" s="1">
@@ -2588,7 +2578,7 @@
       <c r="E93" t="s">
         <v>6</v>
       </c>
-      <c r="I93" s="15"/>
+      <c r="I93" s="18"/>
     </row>
     <row r="94" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A94" s="1">
@@ -2603,22 +2593,25 @@
       <c r="E94" t="s">
         <v>6</v>
       </c>
-      <c r="I94" s="15"/>
+      <c r="I94" s="18"/>
     </row>
     <row r="95" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A95" s="1">
-        <v>24</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>5</v>
+      <c r="A95" s="3">
+        <v>74</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C95" s="13" t="s">
+        <v>68</v>
       </c>
       <c r="D95" s="8">
         <v>96</v>
       </c>
       <c r="E95" t="s">
-        <v>6</v>
-      </c>
-      <c r="I95" s="15"/>
+        <v>14</v>
+      </c>
+      <c r="I95" s="18"/>
     </row>
     <row r="96" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="3">
@@ -2633,7 +2626,7 @@
       <c r="E96" t="s">
         <v>6</v>
       </c>
-      <c r="I96" s="15"/>
+      <c r="I96" s="18"/>
     </row>
     <row r="97" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="3">
@@ -2648,7 +2641,7 @@
       <c r="E97" t="s">
         <v>6</v>
       </c>
-      <c r="I97" s="15"/>
+      <c r="I97" s="18"/>
     </row>
     <row r="98" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="1">
@@ -2666,7 +2659,7 @@
       <c r="E98" t="s">
         <v>1</v>
       </c>
-      <c r="I98" s="15"/>
+      <c r="I98" s="18"/>
     </row>
     <row r="99" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="1">
@@ -2681,7 +2674,7 @@
       <c r="E99" t="s">
         <v>1</v>
       </c>
-      <c r="I99" s="15"/>
+      <c r="I99" s="18"/>
     </row>
     <row r="100" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="1">
@@ -2696,7 +2689,7 @@
       <c r="E100" t="s">
         <v>1</v>
       </c>
-      <c r="I100" s="15"/>
+      <c r="I100" s="18"/>
     </row>
     <row r="101" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="1">
@@ -2711,7 +2704,7 @@
       <c r="E101" t="s">
         <v>1</v>
       </c>
-      <c r="I101" s="15"/>
+      <c r="I101" s="18"/>
     </row>
     <row r="102" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="1">
@@ -2729,7 +2722,7 @@
       <c r="E102" t="s">
         <v>1</v>
       </c>
-      <c r="I102" s="15"/>
+      <c r="I102" s="18"/>
     </row>
     <row r="103" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="2">
@@ -2744,7 +2737,7 @@
       <c r="E103" t="s">
         <v>1</v>
       </c>
-      <c r="I103" s="15"/>
+      <c r="I103" s="18"/>
     </row>
     <row r="104" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="3">
@@ -2759,7 +2752,7 @@
       <c r="E104" t="s">
         <v>1</v>
       </c>
-      <c r="I104" s="15"/>
+      <c r="I104" s="18"/>
     </row>
     <row r="105" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="3">
@@ -2774,7 +2767,7 @@
       <c r="E105" t="s">
         <v>1</v>
       </c>
-      <c r="I105" s="15"/>
+      <c r="I105" s="18"/>
     </row>
     <row r="106" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="3">
@@ -2789,7 +2782,7 @@
       <c r="E106" t="s">
         <v>1</v>
       </c>
-      <c r="I106" s="15"/>
+      <c r="I106" s="18"/>
     </row>
     <row r="107" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A107" s="3">
@@ -2804,7 +2797,7 @@
       <c r="E107" t="s">
         <v>1</v>
       </c>
-      <c r="I107" s="15"/>
+      <c r="I107" s="18"/>
     </row>
     <row r="108" spans="1:9" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A108" s="1">
@@ -2819,7 +2812,7 @@
       <c r="E108" t="s">
         <v>1</v>
       </c>
-      <c r="I108" s="15"/>
+      <c r="I108" s="18"/>
     </row>
     <row r="109" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A109" s="12">
@@ -2834,7 +2827,7 @@
       <c r="E109" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="I109" s="16"/>
+      <c r="I109" s="19"/>
     </row>
     <row r="110" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="1">
@@ -2849,7 +2842,7 @@
       <c r="E110" t="s">
         <v>1</v>
       </c>
-      <c r="I110" s="17" t="s">
+      <c r="I110" s="20" t="s">
         <v>135</v>
       </c>
     </row>
@@ -2866,7 +2859,7 @@
       <c r="E111" t="s">
         <v>1</v>
       </c>
-      <c r="I111" s="18"/>
+      <c r="I111" s="21"/>
     </row>
     <row r="112" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A112" s="2">
@@ -2881,7 +2874,7 @@
       <c r="E112" t="s">
         <v>1</v>
       </c>
-      <c r="I112" s="18"/>
+      <c r="I112" s="21"/>
     </row>
     <row r="113" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A113" s="3">
@@ -2896,7 +2889,7 @@
       <c r="E113" t="s">
         <v>1</v>
       </c>
-      <c r="I113" s="18"/>
+      <c r="I113" s="21"/>
     </row>
     <row r="114" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A114" s="3">
@@ -2911,7 +2904,7 @@
       <c r="E114" t="s">
         <v>1</v>
       </c>
-      <c r="I114" s="18"/>
+      <c r="I114" s="21"/>
     </row>
     <row r="115" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A115" s="3">
@@ -2926,7 +2919,7 @@
       <c r="E115" t="s">
         <v>1</v>
       </c>
-      <c r="I115" s="18"/>
+      <c r="I115" s="21"/>
     </row>
     <row r="116" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="1">
@@ -2941,7 +2934,7 @@
       <c r="E116" t="s">
         <v>1</v>
       </c>
-      <c r="I116" s="18"/>
+      <c r="I116" s="21"/>
     </row>
     <row r="117" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="1">
@@ -2956,7 +2949,7 @@
       <c r="E117" t="s">
         <v>1</v>
       </c>
-      <c r="I117" s="18"/>
+      <c r="I117" s="21"/>
     </row>
     <row r="118" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="1">
@@ -2971,7 +2964,7 @@
       <c r="E118" t="s">
         <v>1</v>
       </c>
-      <c r="I118" s="18"/>
+      <c r="I118" s="21"/>
     </row>
     <row r="119" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="1">
@@ -2986,7 +2979,7 @@
       <c r="E119" t="s">
         <v>1</v>
       </c>
-      <c r="I119" s="18"/>
+      <c r="I119" s="21"/>
     </row>
     <row r="120" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="1">
@@ -3004,7 +2997,7 @@
       <c r="E120" t="s">
         <v>1</v>
       </c>
-      <c r="I120" s="18"/>
+      <c r="I120" s="21"/>
     </row>
     <row r="121" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="1">
@@ -3019,7 +3012,7 @@
       <c r="E121" t="s">
         <v>1</v>
       </c>
-      <c r="I121" s="18"/>
+      <c r="I121" s="21"/>
     </row>
     <row r="122" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="1">
@@ -3034,7 +3027,7 @@
       <c r="E122" t="s">
         <v>1</v>
       </c>
-      <c r="I122" s="18"/>
+      <c r="I122" s="21"/>
     </row>
     <row r="123" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A123" s="1">
@@ -3049,7 +3042,7 @@
       <c r="E123" t="s">
         <v>1</v>
       </c>
-      <c r="I123" s="18"/>
+      <c r="I123" s="21"/>
     </row>
     <row r="124" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="1">
@@ -3067,7 +3060,7 @@
       <c r="E124" t="s">
         <v>1</v>
       </c>
-      <c r="I124" s="18"/>
+      <c r="I124" s="21"/>
     </row>
     <row r="125" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="1">
@@ -3082,7 +3075,7 @@
       <c r="E125" t="s">
         <v>1</v>
       </c>
-      <c r="I125" s="18"/>
+      <c r="I125" s="21"/>
     </row>
     <row r="126" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="2">
@@ -3097,7 +3090,7 @@
       <c r="E126" t="s">
         <v>1</v>
       </c>
-      <c r="I126" s="18"/>
+      <c r="I126" s="21"/>
     </row>
     <row r="127" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="3">
@@ -3112,7 +3105,7 @@
       <c r="E127" t="s">
         <v>1</v>
       </c>
-      <c r="I127" s="18"/>
+      <c r="I127" s="21"/>
     </row>
     <row r="128" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="3">
@@ -3127,7 +3120,7 @@
       <c r="E128" t="s">
         <v>1</v>
       </c>
-      <c r="I128" s="18"/>
+      <c r="I128" s="21"/>
     </row>
     <row r="129" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="3">
@@ -3145,7 +3138,7 @@
       <c r="E129" t="s">
         <v>1</v>
       </c>
-      <c r="I129" s="18"/>
+      <c r="I129" s="21"/>
     </row>
     <row r="130" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="2">
@@ -3160,13 +3153,13 @@
       <c r="E130" t="s">
         <v>1</v>
       </c>
-      <c r="I130" s="18"/>
+      <c r="I130" s="21"/>
     </row>
     <row r="131" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="3">
         <v>6</v>
       </c>
-      <c r="B131" s="21" t="s">
+      <c r="B131" s="3" t="s">
         <v>141</v>
       </c>
       <c r="C131" s="13" t="s">
@@ -3178,13 +3171,13 @@
       <c r="E131" t="s">
         <v>1</v>
       </c>
-      <c r="I131" s="18"/>
+      <c r="I131" s="21"/>
     </row>
     <row r="132" spans="1:9" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="3">
         <v>43</v>
       </c>
-      <c r="B132" s="21" t="s">
+      <c r="B132" s="3" t="s">
         <v>142</v>
       </c>
       <c r="D132" s="8">
@@ -3193,7 +3186,7 @@
       <c r="E132" t="s">
         <v>1</v>
       </c>
-      <c r="I132" s="18"/>
+      <c r="I132" s="21"/>
     </row>
     <row r="133" spans="1:9" s="4" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A133" s="6"/>
@@ -3208,7 +3201,7 @@
       <c r="F133" s="6"/>
       <c r="G133" s="6"/>
       <c r="H133" s="6"/>
-      <c r="I133" s="19"/>
+      <c r="I133" s="22"/>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A135" s="1"/>

</xml_diff>